<commit_message>
Finished full SDD-Dataset validation and added full dataset parser
</commit_message>
<xml_diff>
--- a/data/The-Cancer-Genomic-Atlas/2023-06-29_clean/Clinical Dictionary/GDC_Clinical_CB.xlsx
+++ b/data/The-Cancer-Genomic-Atlas/2023-06-29_clean/Clinical Dictionary/GDC_Clinical_CB.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10611"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10910"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/mjohnson/Projects/SDD-Dataset/data/The-Cancer-Genomic-Atlas/2023-06-29_clean/Clinical Dictionary/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A2D69FCC-5E39-AC4D-8896-E0AC296ACA31}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E5F8D79F-BABD-CD4C-A3B1-01640B7CB45D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="12380" yWindow="8000" windowWidth="27240" windowHeight="16440" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="23620" yWindow="560" windowWidth="27240" windowHeight="16440" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Data Dictionary" sheetId="2" r:id="rId1"/>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="156" uniqueCount="84">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="176" uniqueCount="125">
   <si>
     <t>Gender</t>
   </si>
@@ -273,6 +273,129 @@
   </si>
   <si>
     <t>categorical</t>
+  </si>
+  <si>
+    <t>TARGET USI</t>
+  </si>
+  <si>
+    <t>Age at Diagnosis in Days</t>
+  </si>
+  <si>
+    <t>Time to First Event in Days</t>
+  </si>
+  <si>
+    <t>Overall Survival Time in Days</t>
+  </si>
+  <si>
+    <t>Year of Diagnosis</t>
+  </si>
+  <si>
+    <t>Year of Last Follow Up</t>
+  </si>
+  <si>
+    <t>Protocol</t>
+  </si>
+  <si>
+    <t>Time to first relapse in days</t>
+  </si>
+  <si>
+    <t>Time to first enrollment on relapse protocol in days</t>
+  </si>
+  <si>
+    <t>Time to first SMN in days</t>
+  </si>
+  <si>
+    <t>Time to death in days</t>
+  </si>
+  <si>
+    <t>Histologic response</t>
+  </si>
+  <si>
+    <t>Percent necrosis</t>
+  </si>
+  <si>
+    <t>Relapse Type</t>
+  </si>
+  <si>
+    <t>Therapy</t>
+  </si>
+  <si>
+    <t>Comment</t>
+  </si>
+  <si>
+    <t>string</t>
+  </si>
+  <si>
+    <t>integer</t>
+  </si>
+  <si>
+    <t>date</t>
+  </si>
+  <si>
+    <t>YYYY</t>
+  </si>
+  <si>
+    <t>Subject's age when diagnosed (day)</t>
+  </si>
+  <si>
+    <t>Comments on the subject</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Subject's definitive surgery </t>
+  </si>
+  <si>
+    <t>Subject's disease diagnosis</t>
+  </si>
+  <si>
+    <t>The subject's ethnicity</t>
+  </si>
+  <si>
+    <t>Subject's first event</t>
+  </si>
+  <si>
+    <t>The subject's gender</t>
+  </si>
+  <si>
+    <t>Subject's histologic response range</t>
+  </si>
+  <si>
+    <t>The survival time of the subject (day)</t>
+  </si>
+  <si>
+    <t>The primary tumor's necrosis percentage</t>
+  </si>
+  <si>
+    <t>The primary tumor's site progression</t>
+  </si>
+  <si>
+    <t>The primary tumor's site</t>
+  </si>
+  <si>
+    <t>The subject's race</t>
+  </si>
+  <si>
+    <t>The experimental protocol the subject underwent</t>
+  </si>
+  <si>
+    <t>Subject's relapse type</t>
+  </si>
+  <si>
+    <t>The subject's identifer</t>
+  </si>
+  <si>
+    <t>The therapeutic procedure the subject underwent</t>
+  </si>
+  <si>
+    <t>The subject's vital status</t>
+  </si>
+  <si>
+    <t>The year of diagnosis</t>
+  </si>
+  <si>
+    <t>The first relapse organ site</t>
+  </si>
+  <si>
+    <t>The metastasis growth organ site</t>
   </si>
 </sst>
 </file>
@@ -1157,13 +1280,13 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D8361061-EDFE-6B46-B954-42A1FEC4143A}">
-  <dimension ref="A1:P15"/>
+  <dimension ref="A1:P31"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="21.1640625" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="11.6640625" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="14.33203125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="8.33203125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="44.1640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:16" ht="32" x14ac:dyDescent="0.2">
@@ -1218,23 +1341,32 @@
     </row>
     <row r="2" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
-        <v>0</v>
+        <v>85</v>
+      </c>
+      <c r="D2" t="s">
+        <v>104</v>
       </c>
       <c r="G2" t="s">
-        <v>83</v>
+        <v>101</v>
       </c>
     </row>
     <row r="3" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
-        <v>5</v>
+        <v>99</v>
+      </c>
+      <c r="D3" t="s">
+        <v>105</v>
       </c>
       <c r="G3" t="s">
-        <v>83</v>
+        <v>100</v>
       </c>
     </row>
     <row r="4" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
-        <v>10</v>
+        <v>49</v>
+      </c>
+      <c r="D4" t="s">
+        <v>106</v>
       </c>
       <c r="G4" t="s">
         <v>83</v>
@@ -1242,7 +1374,10 @@
     </row>
     <row r="5" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
-        <v>13</v>
+        <v>21</v>
+      </c>
+      <c r="D5" t="s">
+        <v>107</v>
       </c>
       <c r="G5" t="s">
         <v>83</v>
@@ -1250,7 +1385,10 @@
     </row>
     <row r="6" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
-        <v>18</v>
+        <v>10</v>
+      </c>
+      <c r="D6" t="s">
+        <v>108</v>
       </c>
       <c r="G6" t="s">
         <v>83</v>
@@ -1258,7 +1396,10 @@
     </row>
     <row r="7" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
-        <v>21</v>
+        <v>13</v>
+      </c>
+      <c r="D7" t="s">
+        <v>109</v>
       </c>
       <c r="G7" t="s">
         <v>83</v>
@@ -1266,7 +1407,10 @@
     </row>
     <row r="8" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
-        <v>24</v>
+        <v>0</v>
+      </c>
+      <c r="D8" t="s">
+        <v>110</v>
       </c>
       <c r="G8" t="s">
         <v>83</v>
@@ -1274,15 +1418,21 @@
     </row>
     <row r="9" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
-        <v>28</v>
+        <v>95</v>
+      </c>
+      <c r="D9" t="s">
+        <v>111</v>
       </c>
       <c r="G9" t="s">
-        <v>83</v>
+        <v>100</v>
       </c>
     </row>
     <row r="10" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
-        <v>32</v>
+        <v>24</v>
+      </c>
+      <c r="D10" t="s">
+        <v>124</v>
       </c>
       <c r="G10" t="s">
         <v>83</v>
@@ -1290,23 +1440,32 @@
     </row>
     <row r="11" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
-        <v>43</v>
+        <v>87</v>
+      </c>
+      <c r="D11" t="s">
+        <v>112</v>
       </c>
       <c r="G11" t="s">
-        <v>83</v>
+        <v>101</v>
       </c>
     </row>
     <row r="12" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
-        <v>46</v>
+        <v>96</v>
+      </c>
+      <c r="D12" t="s">
+        <v>113</v>
       </c>
       <c r="G12" t="s">
-        <v>83</v>
+        <v>101</v>
       </c>
     </row>
     <row r="13" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
-        <v>49</v>
+        <v>53</v>
+      </c>
+      <c r="D13" t="s">
+        <v>114</v>
       </c>
       <c r="G13" t="s">
         <v>83</v>
@@ -1314,7 +1473,10 @@
     </row>
     <row r="14" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
-        <v>53</v>
+        <v>28</v>
+      </c>
+      <c r="D14" t="s">
+        <v>115</v>
       </c>
       <c r="G14" t="s">
         <v>83</v>
@@ -1322,13 +1484,201 @@
     </row>
     <row r="15" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
+        <v>90</v>
+      </c>
+      <c r="D15" t="s">
+        <v>117</v>
+      </c>
+      <c r="G15" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="16" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="A16" t="s">
+        <v>5</v>
+      </c>
+      <c r="D16" t="s">
+        <v>116</v>
+      </c>
+      <c r="G16" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="17" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A17" t="s">
+        <v>97</v>
+      </c>
+      <c r="D17" t="s">
+        <v>118</v>
+      </c>
+      <c r="G17" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="18" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A18" t="s">
         <v>56</v>
       </c>
-      <c r="G15" t="s">
+      <c r="D18" t="s">
+        <v>123</v>
+      </c>
+      <c r="G18" t="s">
         <v>83</v>
       </c>
     </row>
+    <row r="19" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A19" t="s">
+        <v>46</v>
+      </c>
+      <c r="D19" t="s">
+        <v>46</v>
+      </c>
+      <c r="G19" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="20" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A20" t="s">
+        <v>43</v>
+      </c>
+      <c r="D20" t="s">
+        <v>43</v>
+      </c>
+      <c r="G20" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="21" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A21" t="s">
+        <v>32</v>
+      </c>
+      <c r="D21" t="s">
+        <v>32</v>
+      </c>
+      <c r="G21" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="22" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A22" t="s">
+        <v>84</v>
+      </c>
+      <c r="D22" t="s">
+        <v>119</v>
+      </c>
+      <c r="G22" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="23" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A23" t="s">
+        <v>98</v>
+      </c>
+      <c r="D23" t="s">
+        <v>120</v>
+      </c>
+      <c r="G23" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="24" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A24" t="s">
+        <v>94</v>
+      </c>
+      <c r="D24" t="s">
+        <v>94</v>
+      </c>
+      <c r="G24" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="25" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A25" t="s">
+        <v>92</v>
+      </c>
+      <c r="D25" t="s">
+        <v>92</v>
+      </c>
+      <c r="G25" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="26" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A26" t="s">
+        <v>86</v>
+      </c>
+      <c r="D26" t="s">
+        <v>86</v>
+      </c>
+      <c r="G26" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="27" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A27" t="s">
+        <v>91</v>
+      </c>
+      <c r="D27" t="s">
+        <v>91</v>
+      </c>
+      <c r="G27" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="28" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A28" t="s">
+        <v>93</v>
+      </c>
+      <c r="D28" t="s">
+        <v>93</v>
+      </c>
+      <c r="G28" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="29" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A29" t="s">
+        <v>18</v>
+      </c>
+      <c r="D29" t="s">
+        <v>121</v>
+      </c>
+      <c r="G29" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="30" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A30" t="s">
+        <v>88</v>
+      </c>
+      <c r="D30" t="s">
+        <v>122</v>
+      </c>
+      <c r="G30" t="s">
+        <v>102</v>
+      </c>
+      <c r="H30" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="31" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A31" t="s">
+        <v>89</v>
+      </c>
+      <c r="D31" t="s">
+        <v>89</v>
+      </c>
+      <c r="G31" t="s">
+        <v>102</v>
+      </c>
+      <c r="H31" t="s">
+        <v>103</v>
+      </c>
+    </row>
   </sheetData>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:P31">
+    <sortCondition ref="A2:A31"/>
+  </sortState>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
@@ -1372,8 +1722,8 @@
       <c r="A2" t="s">
         <v>0</v>
       </c>
-      <c r="C2" t="s">
-        <v>1</v>
+      <c r="C2">
+        <v>0</v>
       </c>
       <c r="D2" t="s">
         <v>1</v>
@@ -1386,8 +1736,8 @@
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="C3" t="s">
-        <v>3</v>
+      <c r="C3">
+        <v>1</v>
       </c>
       <c r="D3" t="s">
         <v>3</v>
@@ -1400,8 +1750,8 @@
       <c r="A4" t="s">
         <v>5</v>
       </c>
-      <c r="C4" t="s">
-        <v>6</v>
+      <c r="C4">
+        <v>0</v>
       </c>
       <c r="D4" t="s">
         <v>6</v>
@@ -1411,24 +1761,24 @@
       </c>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="C5" t="s">
-        <v>7</v>
+      <c r="C5">
+        <v>1</v>
       </c>
       <c r="D5" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="C6" t="s">
-        <v>8</v>
+      <c r="C6">
+        <v>2</v>
       </c>
       <c r="D6" t="s">
         <v>8</v>
       </c>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="C7" t="s">
-        <v>9</v>
+      <c r="C7">
+        <v>3</v>
       </c>
       <c r="D7" t="s">
         <v>9</v>
@@ -1438,8 +1788,8 @@
       <c r="A8" t="s">
         <v>10</v>
       </c>
-      <c r="C8" t="s">
-        <v>11</v>
+      <c r="C8">
+        <v>0</v>
       </c>
       <c r="D8" t="s">
         <v>11</v>
@@ -1449,8 +1799,8 @@
       </c>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="C9" t="s">
-        <v>12</v>
+      <c r="C9">
+        <v>1</v>
       </c>
       <c r="D9" t="s">
         <v>12</v>
@@ -1460,8 +1810,8 @@
       <c r="A10" t="s">
         <v>13</v>
       </c>
-      <c r="C10" t="s">
-        <v>14</v>
+      <c r="C10">
+        <v>0</v>
       </c>
       <c r="D10" t="s">
         <v>14</v>
@@ -1471,24 +1821,24 @@
       </c>
     </row>
     <row r="11" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="C11" t="s">
-        <v>15</v>
+      <c r="C11">
+        <v>1</v>
       </c>
       <c r="D11" t="s">
         <v>15</v>
       </c>
     </row>
     <row r="12" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="C12" t="s">
-        <v>16</v>
+      <c r="C12">
+        <v>2</v>
       </c>
       <c r="D12" t="s">
         <v>16</v>
       </c>
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="C13" t="s">
-        <v>17</v>
+      <c r="C13">
+        <v>3</v>
       </c>
       <c r="D13" t="s">
         <v>17</v>
@@ -1498,8 +1848,8 @@
       <c r="A14" t="s">
         <v>18</v>
       </c>
-      <c r="C14" t="s">
-        <v>19</v>
+      <c r="C14">
+        <v>0</v>
       </c>
       <c r="D14" t="s">
         <v>19</v>
@@ -1509,8 +1859,8 @@
       </c>
     </row>
     <row r="15" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="C15" t="s">
-        <v>20</v>
+      <c r="C15">
+        <v>1</v>
       </c>
       <c r="D15" t="s">
         <v>20</v>
@@ -1520,8 +1870,8 @@
       <c r="A16" t="s">
         <v>21</v>
       </c>
-      <c r="C16" t="s">
-        <v>22</v>
+      <c r="C16">
+        <v>0</v>
       </c>
       <c r="D16" t="s">
         <v>22</v>
@@ -1531,8 +1881,8 @@
       </c>
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="C17" t="s">
-        <v>23</v>
+      <c r="C17">
+        <v>1</v>
       </c>
       <c r="D17" t="s">
         <v>23</v>
@@ -1542,8 +1892,8 @@
       <c r="A18" t="s">
         <v>24</v>
       </c>
-      <c r="C18" t="s">
-        <v>25</v>
+      <c r="C18">
+        <v>0</v>
       </c>
       <c r="D18" t="s">
         <v>25</v>
@@ -1553,16 +1903,16 @@
       </c>
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="C19" t="s">
-        <v>26</v>
+      <c r="C19">
+        <v>1</v>
       </c>
       <c r="D19" t="s">
         <v>26</v>
       </c>
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="C20" t="s">
-        <v>27</v>
+      <c r="C20">
+        <v>2</v>
       </c>
       <c r="D20" t="s">
         <v>27</v>
@@ -1572,8 +1922,8 @@
       <c r="A21" t="s">
         <v>28</v>
       </c>
-      <c r="C21" t="s">
-        <v>29</v>
+      <c r="C21">
+        <v>0</v>
       </c>
       <c r="D21" t="s">
         <v>29</v>
@@ -1583,16 +1933,16 @@
       </c>
     </row>
     <row r="22" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="C22" t="s">
-        <v>30</v>
+      <c r="C22">
+        <v>1</v>
       </c>
       <c r="D22" t="s">
         <v>30</v>
       </c>
     </row>
     <row r="23" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="C23" t="s">
-        <v>31</v>
+      <c r="C23">
+        <v>2</v>
       </c>
       <c r="D23" t="s">
         <v>31</v>
@@ -1602,8 +1952,8 @@
       <c r="A24" t="s">
         <v>32</v>
       </c>
-      <c r="C24" t="s">
-        <v>33</v>
+      <c r="C24">
+        <v>0</v>
       </c>
       <c r="D24" t="s">
         <v>33</v>
@@ -1613,72 +1963,72 @@
       </c>
     </row>
     <row r="25" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="C25" t="s">
-        <v>34</v>
+      <c r="C25">
+        <v>1</v>
       </c>
       <c r="D25" t="s">
         <v>34</v>
       </c>
     </row>
     <row r="26" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="C26" t="s">
-        <v>35</v>
+      <c r="C26">
+        <v>2</v>
       </c>
       <c r="D26" t="s">
         <v>35</v>
       </c>
     </row>
     <row r="27" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="C27" t="s">
-        <v>36</v>
+      <c r="C27">
+        <v>3</v>
       </c>
       <c r="D27" t="s">
         <v>36</v>
       </c>
     </row>
     <row r="28" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="C28" t="s">
-        <v>37</v>
+      <c r="C28">
+        <v>4</v>
       </c>
       <c r="D28" t="s">
         <v>37</v>
       </c>
     </row>
     <row r="29" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="C29" t="s">
-        <v>38</v>
+      <c r="C29">
+        <v>5</v>
       </c>
       <c r="D29" t="s">
         <v>38</v>
       </c>
     </row>
     <row r="30" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="C30" t="s">
-        <v>39</v>
+      <c r="C30">
+        <v>6</v>
       </c>
       <c r="D30" t="s">
         <v>39</v>
       </c>
     </row>
     <row r="31" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="C31" t="s">
-        <v>40</v>
+      <c r="C31">
+        <v>7</v>
       </c>
       <c r="D31" t="s">
         <v>40</v>
       </c>
     </row>
     <row r="32" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="C32" t="s">
-        <v>41</v>
+      <c r="C32">
+        <v>8</v>
       </c>
       <c r="D32" t="s">
         <v>41</v>
       </c>
     </row>
     <row r="33" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="C33" t="s">
-        <v>42</v>
+      <c r="C33">
+        <v>9</v>
       </c>
       <c r="D33" t="s">
         <v>42</v>
@@ -1688,8 +2038,8 @@
       <c r="A34" t="s">
         <v>43</v>
       </c>
-      <c r="C34" t="s">
-        <v>44</v>
+      <c r="C34">
+        <v>0</v>
       </c>
       <c r="D34" t="s">
         <v>44</v>
@@ -1699,8 +2049,8 @@
       </c>
     </row>
     <row r="35" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="C35" t="s">
-        <v>45</v>
+      <c r="C35">
+        <v>1</v>
       </c>
       <c r="D35" t="s">
         <v>45</v>
@@ -1710,8 +2060,8 @@
       <c r="A36" t="s">
         <v>46</v>
       </c>
-      <c r="C36" t="s">
-        <v>47</v>
+      <c r="C36">
+        <v>0</v>
       </c>
       <c r="D36" t="s">
         <v>47</v>
@@ -1721,8 +2071,8 @@
       </c>
     </row>
     <row r="37" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="C37" t="s">
-        <v>48</v>
+      <c r="C37">
+        <v>1</v>
       </c>
       <c r="D37" t="s">
         <v>48</v>
@@ -1732,8 +2082,8 @@
       <c r="A38" t="s">
         <v>49</v>
       </c>
-      <c r="C38" t="s">
-        <v>50</v>
+      <c r="C38">
+        <v>0</v>
       </c>
       <c r="D38" t="s">
         <v>50</v>
@@ -1743,16 +2093,16 @@
       </c>
     </row>
     <row r="39" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="C39" t="s">
-        <v>51</v>
+      <c r="C39">
+        <v>1</v>
       </c>
       <c r="D39" t="s">
         <v>51</v>
       </c>
     </row>
     <row r="40" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="C40" t="s">
-        <v>52</v>
+      <c r="C40">
+        <v>2</v>
       </c>
       <c r="D40" t="s">
         <v>52</v>
@@ -1762,8 +2112,8 @@
       <c r="A41" t="s">
         <v>53</v>
       </c>
-      <c r="C41" t="s">
-        <v>54</v>
+      <c r="C41">
+        <v>0</v>
       </c>
       <c r="D41" t="s">
         <v>54</v>
@@ -1773,8 +2123,8 @@
       </c>
     </row>
     <row r="42" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="C42" t="s">
-        <v>55</v>
+      <c r="C42">
+        <v>1</v>
       </c>
       <c r="D42" t="s">
         <v>55</v>
@@ -1784,8 +2134,8 @@
       <c r="A43" t="s">
         <v>56</v>
       </c>
-      <c r="C43" t="s">
-        <v>25</v>
+      <c r="C43">
+        <v>0</v>
       </c>
       <c r="D43" t="s">
         <v>25</v>
@@ -1795,16 +2145,16 @@
       </c>
     </row>
     <row r="44" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="C44" t="s">
-        <v>57</v>
+      <c r="C44">
+        <v>1</v>
       </c>
       <c r="D44" t="s">
         <v>57</v>
       </c>
     </row>
     <row r="45" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="C45" t="s">
-        <v>58</v>
+      <c r="C45">
+        <v>2</v>
       </c>
       <c r="D45" t="s">
         <v>58</v>

</xml_diff>